<commit_message>
🔧 FIX: Sincronizzazione L0/L1 Stop Loss logic — monitor aggiorna stop_loss_l0_suggested per L0, app.py controlla portfolio_type prima di scegliere colonna
- app.py: Query SELECT include portfolio_type da etf_portfolio_entries
- app.py: _compute_portfolio_sl_positions() controlla portfolio_type prima di leggere stop_loss_l0_suggested vs sl_suggerito
- app.py: result.append() include portfolio_type nell'output JSON
- monitor.py: UPDATE L0 salva sl_suggerito in stop_loss_l0_suggested

Fix completo per l'issue: "Cosa devo fare oggi" vs "Portafoglio" mostravano valori diversi a causa di mischiamento logica L0/L1

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_monitoraggio.xlsx
+++ b/etf_monitoraggio.xlsx
@@ -1993,7 +1993,7 @@
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -8701,7 +8701,7 @@
     </row>
     <row r="98">
       <c r="A98" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -9403,7 +9403,7 @@
     </row>
     <row r="107">
       <c r="A107" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -9481,7 +9481,7 @@
     </row>
     <row r="108">
       <c r="A108" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -12055,7 +12055,7 @@
     </row>
     <row r="141">
       <c r="A141" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -17749,7 +17749,7 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -18763,7 +18763,7 @@
     </row>
     <row r="227">
       <c r="A227" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>

</xml_diff>